<commit_message>
Articles update Krama, JatA and Ghana 12/10/2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Raja Files/Trikrama Table.xlsx
+++ b/TS Jatai Working/Raja Files/Trikrama Table.xlsx
@@ -1,15 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_D04C27874D6FBBFAFDEFC1A7C0FD13475D330168" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -228,7 +240,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -341,9 +353,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -381,9 +393,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -418,7 +430,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -453,7 +465,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -626,7 +638,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:I25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1129,7 +1141,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="B5:F25">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:F25">
     <sortCondition ref="B5:B25"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>